<commit_message>
v2.0.5 - Add format MethodType file excel dau -
</commit_message>
<xml_diff>
--- a/config/Coding/VF3_MHU_F108_v1.xlsx
+++ b/config/Coding/VF3_MHU_F108_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\REDO\CODINGTOOL\config\Coding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24B43018-CC47-4D27-8050-D27F2E277A0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED113FFD-96A6-463D-81F6-8C312994378C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E4BBA423-BD1E-4264-8625-36526A9100A3}"/>
   </bookViews>
@@ -237,23 +237,6 @@
   </si>
   <si>
     <t>CRC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-0x0=Unsupported
-0x1=Vietnamese
-0x2=English
-0x3=Chinese
-0x4=German
-0x5=Russia
-0x6=Japaness
-0x7=Korean
-0x8=French
-0x9=Francais (Canada)
-0xA=Dutch
-0xB=Spanish
-0xC=Hebrew
-0xFF=Invalid</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -833,6 +816,23 @@
 0xFD = Reserved
 0xFE = Reserved
 0xFF = Invalid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+0x0=Unsupported
+0x1 - Vietnamese
+0x2 - English
+0x3=Chinese
+0x4=German
+0x5=Russia
+0x6=Japaness
+0x7=Korean
+0x8=French
+0x9=Francais (Canada)
+0xA=Dutch
+0xB=Spanish
+0xC=Hebrew
+0xFF=Invalid</t>
   </si>
 </sst>
 </file>
@@ -3167,19 +3167,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="10" customFormat="1">
@@ -3233,7 +3233,7 @@
         <v>8</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>49</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="14" customFormat="1" ht="409.6">
@@ -3251,7 +3251,7 @@
         <v>8</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="14" customFormat="1">
@@ -3287,7 +3287,7 @@
         <v>4</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="14" customFormat="1" ht="66">
@@ -3305,7 +3305,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="14" customFormat="1" ht="66">
@@ -3323,7 +3323,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="14" customFormat="1" ht="66">
@@ -3341,7 +3341,7 @@
         <v>2</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="14" customFormat="1" ht="66">
@@ -3359,7 +3359,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="14" customFormat="1" ht="69">
@@ -3377,7 +3377,7 @@
         <v>2</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="1" customFormat="1" ht="66">
@@ -3395,7 +3395,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="1" customFormat="1">
@@ -3431,7 +3431,7 @@
         <v>4</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="1" customFormat="1" ht="409.6">
@@ -3449,7 +3449,7 @@
         <v>8</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="1" customFormat="1">
@@ -3485,7 +3485,7 @@
         <v>2</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="1" customFormat="1" ht="55.2">
@@ -3503,7 +3503,7 @@
         <v>2</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="1" customFormat="1" ht="69">
@@ -3521,7 +3521,7 @@
         <v>2</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="1" customFormat="1" ht="69">
@@ -3539,7 +3539,7 @@
         <v>2</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:6" s="1" customFormat="1" ht="69">
@@ -3557,7 +3557,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:6" s="1" customFormat="1" ht="69">
@@ -3575,7 +3575,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:6" s="1" customFormat="1" ht="110.4">
@@ -3593,7 +3593,7 @@
         <v>4</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="1" customFormat="1" ht="92.4">
@@ -3611,7 +3611,7 @@
         <v>2</v>
       </c>
       <c r="F25" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" spans="1:6" s="1" customFormat="1" ht="66">
@@ -3629,7 +3629,7 @@
         <v>2</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:6" s="1" customFormat="1" ht="96.6">
@@ -3647,7 +3647,7 @@
         <v>2</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:6" s="1" customFormat="1">
@@ -3683,7 +3683,7 @@
         <v>8</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="1" customFormat="1" ht="132">
@@ -3701,7 +3701,7 @@
         <v>8</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31" spans="1:6" s="1" customFormat="1" ht="66">
@@ -3719,7 +3719,7 @@
         <v>2</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:6" s="1" customFormat="1" ht="66">
@@ -3737,7 +3737,7 @@
         <v>2</v>
       </c>
       <c r="F32" s="17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:6" s="1" customFormat="1" ht="66">
@@ -3755,7 +3755,7 @@
         <v>2</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:6" s="1" customFormat="1" ht="92.4">
@@ -3773,7 +3773,7 @@
         <v>2</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:6" s="1" customFormat="1" ht="66">
@@ -3791,7 +3791,7 @@
         <v>2</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36" spans="1:6" s="1" customFormat="1" ht="69">
@@ -3809,7 +3809,7 @@
         <v>2</v>
       </c>
       <c r="F36" s="18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="37" spans="1:6" s="1" customFormat="1" ht="69">
@@ -3827,7 +3827,7 @@
         <v>2</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" spans="1:6" s="1" customFormat="1" ht="69">
@@ -3845,7 +3845,7 @@
         <v>2</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:6" s="1" customFormat="1" ht="55.2">
@@ -3863,7 +3863,7 @@
         <v>2</v>
       </c>
       <c r="F39" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:6" s="1" customFormat="1" ht="69">
@@ -3881,7 +3881,7 @@
         <v>2</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:6" s="1" customFormat="1" ht="82.8">
@@ -3899,7 +3899,7 @@
         <v>2</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:6" s="1" customFormat="1" ht="69">
@@ -3917,7 +3917,7 @@
         <v>2</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:6" s="1" customFormat="1" ht="26.4">

</xml_diff>